<commit_message>
Actualizacion automatica vie 19/06/2026 22:00:02,99
</commit_message>
<xml_diff>
--- a/Jira Tickets GDI.xlsx
+++ b/Jira Tickets GDI.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://intcomexonline-my.sharepoint.com/personal/jpinz390_intcomex_com/Documents/Dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{EDD9222E-5523-4923-98F0-1DF14E60FC75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A6BF929F-3C61-41B5-93A5-99261B89331F}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{EDD9222E-5523-4923-98F0-1DF14E60FC75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F43C89F2-A91E-48DE-AE78-5B26D11134E1}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{4E22F051-163F-463B-B0B3-B9D7B62A7370}"/>
+    <workbookView minimized="1" xWindow="460" yWindow="2300" windowWidth="12800" windowHeight="5680" xr2:uid="{4E22F051-163F-463B-B0B3-B9D7B62A7370}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>

</xml_diff>